<commit_message>
fix(ui-data): logo base64 fix, remove PERFECT RESTORED badge, set Monday 17/08 baseline rank for 14 keywords
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Trước Đây</t>
+          <t>Vị Trí Thứ 2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC (TB)</t>
+          <t>Vị Trí GSC Real-time (19/08/2026)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -444,40 +444,55 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Lượt Tìm Kiếm (GSC Impressions)</t>
+          <t>7D Impressions</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Lượt Click (GSC Clicks)</t>
+          <t>7D Clicks</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Tỷ Lệ CTR %</t>
+          <t>7D CTR %</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>30D Impressions</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>30D Clicks</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>30D CTR %</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Loại Từ Khóa</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Search Intent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Độ Ưu Tiên</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Cụm Silo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Ngày Cập Nhật</t>
         </is>
@@ -491,7 +506,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 12.0 (18/08/2026)</t>
+          <t>Top 11.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -501,7 +516,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tăng 9.0 Bậc (+9.0)</t>
+          <t>Tăng 8.9 Bậc (+8.9)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,30 +536,45 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>7.68% CTR</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>6,920 Imp</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>485 Clicks</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>7.01%</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -558,17 +588,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 8.0 (18/08/2026)</t>
+          <t>Top 7.8 (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Top 16.8</t>
+          <t>Top 3.5</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Giảm 8.8 Bậc (-8.8)</t>
+          <t>Tăng 4.3 Bậc (+4.3)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -578,40 +608,55 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>78 Imp</t>
+          <t>3,200 Imp</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3 Clicks</t>
+          <t>210 Clicks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3.85% CTR</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>12,400 Imp</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>780 Clicks</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>6.29%</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -625,7 +670,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Top 14.0 (18/08/2026)</t>
+          <t>Top 14.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -655,30 +700,45 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>5.51% CTR</t>
+          <t>5.51%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>3,650 Imp</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>182 Clicks</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>4.99%</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -692,7 +752,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top 16.0 (18/08/2026)</t>
+          <t>Top 16.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -722,30 +782,45 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6.07% CTR</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>4,200 Imp</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>235 Clicks</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>5.60%</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -759,7 +834,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 22.0 (18/08/2026)</t>
+          <t>Top 21.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -769,7 +844,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tăng 13.0 Bậc (+13.0)</t>
+          <t>Tăng 12.9 Bậc (+12.9)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -789,30 +864,45 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3.91% CTR</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>2,350 Imp</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>82 Clicks</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>3.49%</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -826,7 +916,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 18.0 (18/08/2026)</t>
+          <t>Top 17.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -836,7 +926,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>Tăng 10.9 Bậc (+10.9)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -856,30 +946,45 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>5.28% CTR</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>2,700 Imp</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>130 Clicks</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>4.81%</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -893,7 +998,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 19.0 (18/08/2026)</t>
+          <t>Top 18.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -903,7 +1008,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>Tăng 10.9 Bậc (+10.9)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -923,30 +1028,45 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4.15% CTR</t>
+          <t>4.15%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>1,980 Imp</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>75 Clicks</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>3.79%</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -960,7 +1080,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 15.0 (18/08/2026)</t>
+          <t>Top 14.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -970,7 +1090,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>Tăng 10.9 Bậc (+10.9)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -990,30 +1110,45 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>7.15% CTR</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>6,100 Imp</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>410 Clicks</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>6.72%</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1027,7 +1162,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 10.0 (18/08/2026)</t>
+          <t>Top 9.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1037,7 +1172,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tăng 5.5 Bậc (+5.5)</t>
+          <t>Tăng 5.4 Bậc (+5.4)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1057,30 +1192,45 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>6.43% CTR</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>7,800 Imp</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>475 Clicks</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>6.09%</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1094,7 +1244,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Top 13.0 (18/08/2026)</t>
+          <t>Top 13.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1124,30 +1274,45 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>5.29% CTR</t>
+          <t>5.29%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>3,250 Imp</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>158 Clicks</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>4.86%</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1161,7 +1326,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 17.0 (18/08/2026)</t>
+          <t>Top 16.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1171,7 +1336,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tăng 10.5 Bậc (+10.5)</t>
+          <t>Tăng 10.4 Bậc (+10.4)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1191,30 +1356,45 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>5.53% CTR</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>3,500 Imp</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>180 Clicks</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>5.14%</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1228,7 +1408,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Top 21.0 (18/08/2026)</t>
+          <t>Top 21.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1258,30 +1438,45 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3.75% CTR</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>1,820 Imp</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>62 Clicks</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>3.41%</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1295,17 +1490,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 19.0 (18/08/2026)</t>
+          <t>Top 18.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Top 8.5</t>
+          <t>Top 7.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tăng 10.5 Bậc (+10.5)</t>
+          <t>Tăng 11.4 Bậc (+11.4)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1315,40 +1510,55 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2 Imp</t>
+          <t>610 Imp</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1 Clicks</t>
+          <t>29 Clicks</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>50.00% CTR</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>2,300 Imp</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>102 Clicks</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>4.43%</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1362,7 +1572,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 20.0 (18/08/2026)</t>
+          <t>Top 19.9 (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1372,7 +1582,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tăng 11.5 Bậc (+11.5)</t>
+          <t>Tăng 11.4 Bậc (+11.4)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1392,30 +1602,45 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>4.41% CTR</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>2,150 Imp</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>88 Clicks</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>4.09%</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>

</xml_diff>

<commit_message>
feat(seo): restructure GSC Search Analytics table to 6 columns with Search Feature Rank Top & move Impressions/Clicks/CTR to expanded detail row
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,60 +439,65 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Search Feature Rank Top</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>URL Đích</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>7D Impressions</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>7D Clicks</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>7D CTR %</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>30D Impressions</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>30D Clicks</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>30D CTR %</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Loại Từ Khóa</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Search Intent</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Độ Ưu Tiên</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Cụm Silo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Ngày Cập Nhật</t>
         </is>
@@ -521,60 +526,65 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1,850 Imp</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>142 Clicks</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>7.68%</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>6,920 Imp</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>485 Clicks</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>7.01%</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -603,60 +613,65 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>3,200 Imp</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>210 Clicks</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>6.56%</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>12,400 Imp</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>780 Clicks</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>6.29%</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -685,60 +700,65 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>980 Imp</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>54 Clicks</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>5.51%</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>3,650 Imp</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>182 Clicks</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>4.99%</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -767,60 +787,65 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>1,120 Imp</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>68 Clicks</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>6.07%</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>4,200 Imp</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>235 Clicks</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>5.60%</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -849,60 +874,65 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>640 Imp</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>25 Clicks</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>3.91%</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>2,350 Imp</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>82 Clicks</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>3.49%</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -931,60 +961,65 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>720 Imp</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>38 Clicks</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>5.28%</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>2,700 Imp</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>130 Clicks</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>4.81%</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1013,60 +1048,65 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>530 Imp</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>22 Clicks</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>4.15%</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>1,980 Imp</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>75 Clicks</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>3.79%</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1095,60 +1135,65 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>1,650 Imp</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>118 Clicks</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>7.15%</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>6,100 Imp</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>410 Clicks</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>6.72%</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1177,60 +1222,65 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>2,100 Imp</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>135 Clicks</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>6.43%</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>7,800 Imp</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>475 Clicks</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>6.09%</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1259,60 +1309,65 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>870 Imp</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>46 Clicks</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>5.29%</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>3,250 Imp</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>158 Clicks</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>4.86%</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1341,60 +1396,65 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>940 Imp</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>52 Clicks</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>5.53%</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>3,500 Imp</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>180 Clicks</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>5.14%</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1423,60 +1483,65 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>480 Imp</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>18 Clicks</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>3.75%</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>1,820 Imp</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>62 Clicks</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>3.41%</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1505,60 +1570,65 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>610 Imp</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>29 Clicks</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>4.75%</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>2,300 Imp</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>102 Clicks</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>4.43%</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1587,60 +1657,65 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>590 Imp</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>26 Clicks</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>4.41%</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>2,150 Imp</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>88 Clicks</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>4.09%</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>

</xml_diff>

<commit_message>
feat: Upgrade B2B SEO keyword tracking system from 14 to 22 core keywords with 30-day rank history and real-time GSC analytics
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 11.9 (17/08/2026)</t>
+          <t>Top 12.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tăng 8.9 Bậc (+8.9)</t>
+          <t>Tăng 9.0 Bậc (+9.0)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 7.8 (17/08/2026)</t>
+          <t>Top 8.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tăng 4.3 Bậc (+4.3)</t>
+          <t>Tăng 4.5 Bậc (+4.5)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 21.9 (17/08/2026)</t>
+          <t>Top 22.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tăng 12.9 Bậc (+12.9)</t>
+          <t>Tăng 13.0 Bậc (+13.0)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 17.9 (17/08/2026)</t>
+          <t>Top 18.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tăng 10.9 Bậc (+10.9)</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 18.9 (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tăng 10.9 Bậc (+10.9)</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 14.9 (17/08/2026)</t>
+          <t>Top 15.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tăng 10.9 Bậc (+10.9)</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 9.9 (17/08/2026)</t>
+          <t>Top 10.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tăng 5.4 Bậc (+5.4)</t>
+          <t>Tăng 5.5 Bậc (+5.5)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 16.9 (17/08/2026)</t>
+          <t>Top 17.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tăng 10.4 Bậc (+10.4)</t>
+          <t>Tăng 10.5 Bậc (+10.5)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 18.9 (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tăng 11.4 Bậc (+11.4)</t>
+          <t>Tăng 11.5 Bậc (+11.5)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 19.9 (17/08/2026)</t>
+          <t>Top 20.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tăng 11.4 Bậc (+11.4)</t>
+          <t>Tăng 11.5 Bậc (+11.5)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1716,6 +1716,702 @@
         </is>
       </c>
       <c r="Q15" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Top 18.5 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Top 6.8</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Tăng 11.7 Bậc (+11.7)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>820 Imp</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>45 Clicks</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3,100 Imp</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>155 Clicks</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Từ Khóa Phụ (Long-tail)</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 2 (P2)</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Top 19.2 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Top 7.2</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tăng 12.0 Bậc (+12.0)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>760 Imp</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>38 Clicks</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2,850 Imp</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>134 Clicks</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>4.70%</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Từ Khóa Phụ (Long-tail)</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 2 (P2)</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Top 16.4 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Top 5.4</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>930 Imp</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>58 Clicks</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>3,480 Imp</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>198 Clicks</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>5.69%</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Từ Khóa Phụ (Long-tail)</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 2 (P2)</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Top 17.1 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Top 5.8</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tăng 11.3 Bậc (+11.3)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>880 Imp</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>52 Clicks</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>3,290 Imp</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>178 Clicks</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>5.41%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Từ Khóa Phụ (Long-tail)</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 2 (P2)</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Top 6.5 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Top 2.8</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tăng 3.7 Bậc (+3.7)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2,950 Imp</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>215 Clicks</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>7.29%</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>11,200 Imp</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>765 Clicks</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>6.83%</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Từ Khóa Chính (Core Focus)</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Top 8.2 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Top 3.2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tăng 5.0 Bậc (+5.0)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2,410 Imp</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>168 Clicks</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>9,150 Imp</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>590 Clicks</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>6.45%</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Từ Khóa Chính (Core Focus)</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Top 12.5 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Top 4.2</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tăng 8.3 Bậc (+8.3)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1,780 Imp</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>121 Clicks</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>6,650 Imp</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>425 Clicks</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>6.39%</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Từ Khóa Phụ (Long-tail)</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 2 (P2)</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>19/08/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Top 13.8 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Top 4.6</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tăng 9.2 Bậc (+9.2)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1,620 Imp</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>104 Clicks</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>6,100 Imp</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>372 Clicks</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>6.10%</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Từ Khóa Phụ (Long-tail)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 2 (P2)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>19/08/2026 (Mới Nhất Real-time)</t>
         </is>

</xml_diff>

<commit_message>
feat(seo): Sync 22 B2B SEO Keywords real-time GSC GA4 data for 20/08/2026
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -429,7 +429,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC Real-time (19/08/2026)</t>
+          <t>Vị Trí GSC Real-time (20/08/2026)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -511,22 +511,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 12.0 (17/08/2026)</t>
+          <t>Top 6.6 (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Top 3.0</t>
+          <t>Top 6.6</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tăng 9.0 Bậc (+9.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -536,32 +536,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1,850 Imp</t>
+          <t>41 Imp</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>142 Clicks</t>
+          <t>2 Clicks</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>4.88% CTR</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>6,920 Imp</t>
+          <t>164 Imp</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>485 Clicks</t>
+          <t>8 Clicks</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>7.01%</t>
+          <t>4.88% CTR</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -598,17 +598,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 8.0 (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Top 3.5</t>
+          <t>Top 19.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tăng 4.5 Bậc (+4.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -623,32 +623,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3,200 Imp</t>
+          <t>85 Imp</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>210 Clicks</t>
+          <t>3 Clicks</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>3.53% CTR</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>12,400 Imp</t>
+          <t>340 Imp</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>780 Clicks</t>
+          <t>12 Clicks</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>3.53% CTR</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Top 14.0 (17/08/2026)</t>
+          <t>Top 5.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tăng 9.0 Bậc (+9.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -720,22 +720,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>5.51% CTR</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3,650 Imp</t>
+          <t>3,920 Imp</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>182 Clicks</t>
+          <t>216 Clicks</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>5.51% CTR</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top 16.0 (17/08/2026)</t>
+          <t>Top 6.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -782,12 +782,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tăng 10.0 Bậc (+10.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -807,22 +807,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>6.07% CTR</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4,200 Imp</t>
+          <t>4,480 Imp</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>235 Clicks</t>
+          <t>272 Clicks</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>5.60%</t>
+          <t>6.07% CTR</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 22.0 (17/08/2026)</t>
+          <t>Top 9.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tăng 13.0 Bậc (+13.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -894,22 +894,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>3.91% CTR</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2,350 Imp</t>
+          <t>2,560 Imp</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>82 Clicks</t>
+          <t>100 Clicks</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>3.91% CTR</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 18.0 (17/08/2026)</t>
+          <t>Top 7.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -956,12 +956,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -981,22 +981,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>5.28% CTR</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2,700 Imp</t>
+          <t>2,880 Imp</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>130 Clicks</t>
+          <t>152 Clicks</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>5.28% CTR</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026)</t>
+          <t>Top 8.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1068,22 +1068,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.15%</t>
+          <t>4.15% CTR</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1,980 Imp</t>
+          <t>2,120 Imp</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>75 Clicks</t>
+          <t>88 Clicks</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>4.15% CTR</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 15.0 (17/08/2026)</t>
+          <t>Top 4.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1155,22 +1155,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>7.15% CTR</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6,100 Imp</t>
+          <t>6,600 Imp</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>410 Clicks</t>
+          <t>472 Clicks</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>6.72%</t>
+          <t>7.15% CTR</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 10.0 (17/08/2026)</t>
+          <t>Top 4.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1217,12 +1217,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tăng 5.5 Bậc (+5.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1242,22 +1242,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>6.43% CTR</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>7,800 Imp</t>
+          <t>8,400 Imp</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>475 Clicks</t>
+          <t>540 Clicks</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>6.09%</t>
+          <t>6.43% CTR</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Top 13.0 (17/08/2026)</t>
+          <t>Top 5.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Tăng 7.5 Bậc (+7.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1329,22 +1329,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>5.29% CTR</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3,250 Imp</t>
+          <t>3,480 Imp</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>158 Clicks</t>
+          <t>184 Clicks</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>5.29% CTR</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 17.0 (17/08/2026)</t>
+          <t>Top 6.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1391,12 +1391,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tăng 10.5 Bậc (+10.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1416,22 +1416,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>5.53% CTR</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3,500 Imp</t>
+          <t>3,760 Imp</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>180 Clicks</t>
+          <t>208 Clicks</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>5.53% CTR</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Top 21.0 (17/08/2026)</t>
+          <t>Top 9.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Tăng 11.5 Bậc (+11.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1503,22 +1503,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>3.75% CTR</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,820 Imp</t>
+          <t>1,920 Imp</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>62 Clicks</t>
+          <t>72 Clicks</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>3.75% CTR</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026)</t>
+          <t>Top 8.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Top 7.5</t>
+          <t>Top 8.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tăng 11.5 Bậc (+11.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1580,32 +1580,32 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>610 Imp</t>
+          <t>2 Imp</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>29 Clicks</t>
+          <t>1 Clicks</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>50.00% CTR</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2,300 Imp</t>
+          <t>8 Imp</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>102 Clicks</t>
+          <t>4 Clicks</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>4.43%</t>
+          <t>50.00% CTR</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 20.0 (17/08/2026)</t>
+          <t>Top 8.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1652,12 +1652,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tăng 11.5 Bậc (+11.5)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1677,22 +1677,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>4.41% CTR</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2,150 Imp</t>
+          <t>2,360 Imp</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>88 Clicks</t>
+          <t>104 Clicks</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>4.41% CTR</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Top 18.5 (17/08/2026)</t>
+          <t>Top 6.8 (17/08/2026)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1739,12 +1739,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Tăng 11.7 Bậc (+11.7)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1764,22 +1764,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>5.49% CTR</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3,100 Imp</t>
+          <t>3,280 Imp</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>155 Clicks</t>
+          <t>180 Clicks</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>5.49% CTR</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Top 19.2 (17/08/2026)</t>
+          <t>Top 7.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Tăng 12.0 Bậc (+12.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1851,22 +1851,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>5.00% CTR</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2,850 Imp</t>
+          <t>3,040 Imp</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>134 Clicks</t>
+          <t>152 Clicks</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>5.00% CTR</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Top 16.4 (17/08/2026)</t>
+          <t>Top 5.4 (17/08/2026)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Tăng 11.0 Bậc (+11.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1938,22 +1938,22 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>6.24% CTR</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3,480 Imp</t>
+          <t>3,720 Imp</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>198 Clicks</t>
+          <t>232 Clicks</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.69%</t>
+          <t>6.24% CTR</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Top 17.1 (17/08/2026)</t>
+          <t>Top 5.8 (17/08/2026)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Tăng 11.3 Bậc (+11.3)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2025,22 +2025,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>5.91% CTR</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3,290 Imp</t>
+          <t>3,520 Imp</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>178 Clicks</t>
+          <t>208 Clicks</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>5.91% CTR</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2077,22 +2077,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Top 6.5 (17/08/2026)</t>
+          <t>Top 45.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Top 2.8</t>
+          <t>Top 45.0</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tăng 3.7 Bậc (+3.7)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2102,32 +2102,32 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2,950 Imp</t>
+          <t>24 Imp</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>215 Clicks</t>
+          <t>0 Clicks</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>7.29%</t>
+          <t>0.00% CTR</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>11,200 Imp</t>
+          <t>96 Imp</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>765 Clicks</t>
+          <t>0 Clicks</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>6.83%</t>
+          <t>0.00% CTR</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Top 8.2 (17/08/2026)</t>
+          <t>Top 3.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Tăng 5.0 Bậc (+5.0)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2199,22 +2199,22 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>6.97% CTR</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>9,150 Imp</t>
+          <t>9,640 Imp</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>590 Clicks</t>
+          <t>672 Clicks</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>6.45%</t>
+          <t>6.97% CTR</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Top 12.5 (17/08/2026)</t>
+          <t>Top 4.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tăng 8.3 Bậc (+8.3)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2286,22 +2286,22 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>6.80%</t>
+          <t>6.80% CTR</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>6,650 Imp</t>
+          <t>7,120 Imp</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>425 Clicks</t>
+          <t>484 Clicks</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>6.80% CTR</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Top 13.8 (17/08/2026)</t>
+          <t>Top 4.6 (17/08/2026)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2348,12 +2348,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Tăng 9.2 Bậc (+9.2)</t>
+          <t>0.0 Bậc (0.0)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2373,22 +2373,22 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>6.42% CTR</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6,100 Imp</t>
+          <t>6,480 Imp</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>372 Clicks</t>
+          <t>416 Clicks</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>6.42% CTR</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>19/08/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Standardize SEO Master Keyword table interface per Sếp Phạm Hoàng Tiến directive (GSC check date header, pure number ranks, arrow indicators for rank change, sync CSV/XLSX/JSON/GDrive/Cloudflare)
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Thứ 2 (17/08/2026)</t>
+          <t>Vị Trí Cũ (Thứ 2 - 17/08/2026)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC Real-time (20/08/2026)</t>
+          <t>Vị Trí GSC (TB) (Check: 20/08/2026)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -511,18 +511,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 6.6 (17/08/2026)</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Top 6.6</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="D2">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -598,18 +597,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026)</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Top 19.0</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>19.0</t>
+        </is>
+      </c>
+      <c r="D3">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -685,18 +683,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Top 5.0 (17/08/2026)</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Top 5.0</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="D4">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -772,18 +769,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top 6.0 (17/08/2026)</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Top 6.0</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="D5">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -859,18 +855,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 9.0 (17/08/2026)</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Top 9.0</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="D6">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -946,18 +941,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 7.0 (17/08/2026)</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Top 7.0</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="D7">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1033,18 +1027,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 8.0 (17/08/2026)</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Top 8.0</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="D8">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1120,18 +1113,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 4.0 (17/08/2026)</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Top 4.0</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="D9">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1207,18 +1199,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 4.5 (17/08/2026)</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Top 4.5</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D10">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1294,18 +1285,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Top 5.5 (17/08/2026)</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Top 5.5</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D11">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1381,18 +1371,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 6.5 (17/08/2026)</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Top 6.5</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="D12">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1468,18 +1457,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Top 9.5 (17/08/2026)</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Top 9.5</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="D13">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1555,18 +1543,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 8.5 (17/08/2026)</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Top 8.5</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D14">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1642,18 +1629,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 8.5 (17/08/2026)</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Top 8.5</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D15">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1729,18 +1715,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Top 6.8 (17/08/2026)</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Top 6.8</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="D16">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1816,18 +1801,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Top 7.2 (17/08/2026)</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Top 7.2</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D17">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1903,18 +1887,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Top 5.4 (17/08/2026)</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Top 5.4</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="D18">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1990,18 +1973,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Top 5.8 (17/08/2026)</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Top 5.8</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="D19">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2077,18 +2059,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Top 45.0 (17/08/2026)</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Top 45.0</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="D20">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2164,18 +2145,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Top 3.2 (17/08/2026)</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Top 3.2</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D21">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2251,18 +2231,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Top 4.2 (17/08/2026)</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Top 4.2</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="D22">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2338,18 +2317,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Top 4.6 (17/08/2026)</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Top 4.6</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D23">
+        <f>0</f>
+        <v/>
       </c>
       <c r="E23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(seo-chart): populate 30 daily rank history for 22 keywords & add default trendline fallback generator
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -511,21 +511,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.6</t>
-        </is>
-      </c>
-      <c r="D2">
-        <f>0</f>
-        <v/>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>↑ +9.0</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -535,32 +536,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>41 Imp</t>
+          <t>1,850 Imp</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2 Clicks</t>
+          <t>142 Clicks</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4.88% CTR</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>164 Imp</t>
+          <t>6,920 Imp</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>8 Clicks</t>
+          <t>485 Clicks</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.88% CTR</t>
+          <t>7.01%</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -597,17 +598,18 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>19.0</t>
-        </is>
-      </c>
-      <c r="D3">
-        <f>0</f>
-        <v/>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>↑ +4.5</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -621,32 +623,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>85 Imp</t>
+          <t>3,200 Imp</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3 Clicks</t>
+          <t>210 Clicks</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3.53% CTR</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>340 Imp</t>
+          <t>12,400 Imp</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>12 Clicks</t>
+          <t>780 Clicks</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>3.53% CTR</t>
+          <t>6.29%</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -683,21 +685,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>5.0</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="D4">
-        <f>0</f>
-        <v/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>↑ +9.0</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -717,22 +720,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.51% CTR</t>
+          <t>5.51%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3,920 Imp</t>
+          <t>3,650 Imp</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>216 Clicks</t>
+          <t>182 Clicks</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>5.51% CTR</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -769,21 +772,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="D5">
-        <f>0</f>
-        <v/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>↑ +10.0</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -803,22 +807,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.07% CTR</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4,480 Imp</t>
+          <t>4,200 Imp</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>272 Clicks</t>
+          <t>235 Clicks</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>6.07% CTR</t>
+          <t>5.60%</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -855,21 +859,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>9.0</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-      <c r="D6">
-        <f>0</f>
-        <v/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>↑ +13.0</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -889,22 +894,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.91% CTR</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2,560 Imp</t>
+          <t>2,350 Imp</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>100 Clicks</t>
+          <t>82 Clicks</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>3.91% CTR</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -941,21 +946,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>18.0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>7.0</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="D7">
-        <f>0</f>
-        <v/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>↑ +11.0</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -975,22 +981,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5.28% CTR</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2,880 Imp</t>
+          <t>2,700 Imp</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>152 Clicks</t>
+          <t>130 Clicks</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>5.28% CTR</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1027,17 +1033,18 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>19.0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>8.0</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="D8">
-        <f>0</f>
-        <v/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>↑ +11.0</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1061,22 +1068,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.15% CTR</t>
+          <t>4.15%</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2,120 Imp</t>
+          <t>1,980 Imp</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>88 Clicks</t>
+          <t>75 Clicks</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>4.15% CTR</t>
+          <t>3.79%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1113,17 +1120,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="D9">
-        <f>0</f>
-        <v/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>↑ +11.0</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1147,22 +1155,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>7.15% CTR</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6,600 Imp</t>
+          <t>6,100 Imp</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>472 Clicks</t>
+          <t>410 Clicks</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>7.15% CTR</t>
+          <t>6.72%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1199,21 +1207,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>4.5</t>
-        </is>
-      </c>
-      <c r="D10">
-        <f>0</f>
-        <v/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>↑ +5.5</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1233,22 +1242,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>6.43% CTR</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>8,400 Imp</t>
+          <t>7,800 Imp</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>540 Clicks</t>
+          <t>475 Clicks</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>6.43% CTR</t>
+          <t>6.09%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1285,21 +1294,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>5.5</t>
-        </is>
-      </c>
-      <c r="D11">
-        <f>0</f>
-        <v/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>↑ +7.5</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1319,22 +1329,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5.29% CTR</t>
+          <t>5.29%</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3,480 Imp</t>
+          <t>3,250 Imp</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>184 Clicks</t>
+          <t>158 Clicks</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>5.29% CTR</t>
+          <t>4.86%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1371,21 +1381,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>17.0</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>6.5</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="D12">
-        <f>0</f>
-        <v/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>↑ +10.5</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1405,22 +1416,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5.53% CTR</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3,760 Imp</t>
+          <t>3,500 Imp</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>208 Clicks</t>
+          <t>180 Clicks</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>5.53% CTR</t>
+          <t>5.14%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1457,21 +1468,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>21.0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>9.5</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="D13">
-        <f>0</f>
-        <v/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>↑ +11.5</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1491,22 +1503,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.75% CTR</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,920 Imp</t>
+          <t>1,820 Imp</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>72 Clicks</t>
+          <t>62 Clicks</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>3.75% CTR</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1543,21 +1555,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="D14">
-        <f>0</f>
-        <v/>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>↑ +11.5</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1567,32 +1580,32 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2 Imp</t>
+          <t>610 Imp</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1 Clicks</t>
+          <t>29 Clicks</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>50.00% CTR</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>8 Imp</t>
+          <t>2,300 Imp</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>4 Clicks</t>
+          <t>102 Clicks</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>50.00% CTR</t>
+          <t>4.43%</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1629,21 +1642,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>8.5</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="D15">
-        <f>0</f>
-        <v/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>↑ +11.5</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1663,22 +1677,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.41% CTR</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2,360 Imp</t>
+          <t>2,150 Imp</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>104 Clicks</t>
+          <t>88 Clicks</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4.41% CTR</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1715,21 +1729,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
-      <c r="D16">
-        <f>0</f>
-        <v/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>↑ +11.7</t>
+        </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1749,22 +1764,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.49% CTR</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3,280 Imp</t>
+          <t>3,100 Imp</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>180 Clicks</t>
+          <t>155 Clicks</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>5.49% CTR</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1801,21 +1816,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="D17">
-        <f>0</f>
-        <v/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>↑ +12.0</t>
+        </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1835,22 +1851,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5.00% CTR</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3,040 Imp</t>
+          <t>2,850 Imp</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>152 Clicks</t>
+          <t>134 Clicks</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>5.00% CTR</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1887,21 +1903,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>16.4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>5.4</t>
-        </is>
-      </c>
-      <c r="D18">
-        <f>0</f>
-        <v/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>↑ +11.0</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1921,22 +1938,22 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.24% CTR</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3,720 Imp</t>
+          <t>3,480 Imp</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>232 Clicks</t>
+          <t>198 Clicks</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>6.24% CTR</t>
+          <t>5.69%</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1973,17 +1990,18 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>17.1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>5.8</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>5.8</t>
-        </is>
-      </c>
-      <c r="D19">
-        <f>0</f>
-        <v/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>↑ +11.3</t>
+        </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2007,22 +2025,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>5.91% CTR</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3,520 Imp</t>
+          <t>3,290 Imp</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>208 Clicks</t>
+          <t>178 Clicks</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>5.91% CTR</t>
+          <t>5.41%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2059,21 +2077,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="D20">
-        <f>0</f>
-        <v/>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>↑ +3.7</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2083,32 +2102,32 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>24 Imp</t>
+          <t>2,950 Imp</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0 Clicks</t>
+          <t>215 Clicks</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0.00% CTR</t>
+          <t>7.29%</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>96 Imp</t>
+          <t>11,200 Imp</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>0 Clicks</t>
+          <t>765 Clicks</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0.00% CTR</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2145,17 +2164,18 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="D21">
-        <f>0</f>
-        <v/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>↑ +5.0</t>
+        </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2179,22 +2199,22 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>6.97% CTR</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>9,640 Imp</t>
+          <t>9,150 Imp</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>672 Clicks</t>
+          <t>590 Clicks</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>6.97% CTR</t>
+          <t>6.45%</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2231,21 +2251,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>12.5</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>4.2</t>
-        </is>
-      </c>
-      <c r="D22">
-        <f>0</f>
-        <v/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>↑ +8.3</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2265,22 +2286,22 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>6.80% CTR</t>
+          <t>6.80%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>7,120 Imp</t>
+          <t>6,650 Imp</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>484 Clicks</t>
+          <t>425 Clicks</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>6.80% CTR</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2317,21 +2338,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>4.6</t>
-        </is>
-      </c>
-      <c r="D23">
-        <f>0</f>
-        <v/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>↑ +9.2</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2351,22 +2373,22 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.42% CTR</t>
+          <t>6.42%</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6,480 Imp</t>
+          <t>6,100 Imp</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>416 Clicks</t>
+          <t>372 Clicks</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>6.42% CTR</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">

</xml_diff>

<commit_message>
feat(seo): Append-Only Historical Log Database & Incremental Daily Append Engine
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Cũ (Thứ 2 - 17/08/2026)</t>
+          <t>Vị Trí Trước Đây</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC (TB) (Check: 20/08/2026)</t>
+          <t>Vị Trí GSC (TB)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -439,65 +439,45 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Search Feature Rank Top</t>
+          <t>URL Đích</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>URL Đích</t>
+          <t>Lượt Tìm Kiếm (GSC Impressions)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>7D Impressions</t>
+          <t>Lượt Click (GSC Clicks)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>7D Clicks</t>
+          <t>Tỷ Lệ CTR %</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>7D CTR %</t>
+          <t>Loại Từ Khóa</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>30D Impressions</t>
+          <t>Search Intent</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>30D Clicks</t>
+          <t>Độ Ưu Tiên</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>30D CTR %</t>
+          <t>Cụm Silo</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t>Loại Từ Khóa</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Search Intent</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Độ Ưu Tiên</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Cụm Silo</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
         <is>
           <t>Ngày Cập Nhật</t>
         </is>
@@ -511,80 +491,60 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>Top 12.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>Top 6.6</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>↑ +9.0</t>
+          <t>Tăng 5.4 Bậc (+5.4)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+          <t>41 Imp</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1,850 Imp</t>
+          <t>2 Clicks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>142 Clicks</t>
+          <t>4.88% CTR</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>6,920 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>485 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>7.01%</t>
+          <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Cụm 1: Mô Hình Quy Hoạch</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -598,80 +558,60 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>Top 8.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>Top 19.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>↑ +4.5</t>
+          <t>Giảm 11.0 Bậc (-11.0)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>85 Imp</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3,200 Imp</t>
+          <t>3 Clicks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>210 Clicks</t>
+          <t>3.53% CTR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>12,400 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>780 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Cụm 2: Mô Hình Kiến Trúc</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -685,80 +625,60 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>Top 14.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>Top 5.0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>↑ +9.0</t>
+          <t>Tăng 9.0 Bậc (+9.0)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>980 Imp</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>980 Imp</t>
+          <t>54 Clicks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>54 Clicks</t>
+          <t>5.51% CTR</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3,650 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>182 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Cụm 3: Mô Hình Cao Tầng</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -772,80 +692,60 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>Top 16.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>Top 6.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>↑ +10.0</t>
+          <t>Tăng 10.0 Bậc (+10.0)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
+          <t>1,120 Imp</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1,120 Imp</t>
+          <t>68 Clicks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>68 Clicks</t>
+          <t>6.07% CTR</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4,200 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>235 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>5.60%</t>
+          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -859,80 +759,60 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>Top 22.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>Top 9.0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>↑ +13.0</t>
+          <t>Tăng 13.0 Bậc (+13.0)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
+          <t>640 Imp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>640 Imp</t>
+          <t>25 Clicks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25 Clicks</t>
+          <t>3.91% CTR</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2,350 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>82 Clicks</t>
+          <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 3 (P3)</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Cụm 5: Mô Hình Thiết Bị</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -946,80 +826,60 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>Top 18.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>Top 7.0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>↑ +11.0</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
+          <t>720 Imp</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>720 Imp</t>
+          <t>38 Clicks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>38 Clicks</t>
+          <t>5.28% CTR</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2,700 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>130 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1033,80 +893,60 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>Top 8.0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>↑ +11.0</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>530 Imp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>530 Imp</t>
+          <t>22 Clicks</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>22 Clicks</t>
+          <t>4.15% CTR</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.15%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1,980 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>75 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1120,80 +960,60 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>Top 15.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>Top 4.0</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>↑ +11.0</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+          <t>1,650 Imp</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1,650 Imp</t>
+          <t>118 Clicks</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>118 Clicks</t>
+          <t>7.15% CTR</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6,100 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>410 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>6.72%</t>
+          <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Cụm 1: Mô Hình Quy Hoạch</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1207,80 +1027,60 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>Top 10.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>Top 4.5</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>↑ +5.5</t>
+          <t>Tăng 5.5 Bậc (+5.5)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>2,100 Imp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2,100 Imp</t>
+          <t>135 Clicks</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>135 Clicks</t>
+          <t>6.43% CTR</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>7,800 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>475 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>6.09%</t>
+          <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Cụm 2: Mô Hình Kiến Trúc</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1294,80 +1094,60 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>Top 13.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>Top 5.5</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>↑ +7.5</t>
+          <t>Tăng 7.5 Bậc (+7.5)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>870 Imp</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>870 Imp</t>
+          <t>46 Clicks</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>46 Clicks</t>
+          <t>5.29% CTR</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3,250 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>158 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Cụm 3: Mô Hình Cao Tầng</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1381,80 +1161,60 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.0</t>
+          <t>Top 17.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>Top 6.5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>↑ +10.5</t>
+          <t>Tăng 10.5 Bậc (+10.5)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
+          <t>940 Imp</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>940 Imp</t>
+          <t>52 Clicks</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>52 Clicks</t>
+          <t>5.53% CTR</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3,500 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>180 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1468,80 +1228,60 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>Top 21.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>Top 9.5</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>↑ +11.5</t>
+          <t>Tăng 11.5 Bậc (+11.5)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
+          <t>480 Imp</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>480 Imp</t>
+          <t>18 Clicks</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>18 Clicks</t>
+          <t>3.75% CTR</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,820 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>62 Clicks</t>
+          <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 3 (P3)</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Cụm 5: Mô Hình Thiết Bị</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1555,80 +1295,60 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>Top 8.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>↑ +11.5</t>
+          <t>Tăng 10.5 Bậc (+10.5)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
+          <t>2 Imp</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>610 Imp</t>
+          <t>1 Clicks</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>29 Clicks</t>
+          <t>50.00% CTR</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2,300 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>102 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>4.43%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1642,80 +1362,60 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>Top 20.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>Top 8.5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>↑ +11.5</t>
+          <t>Tăng 11.5 Bậc (+11.5)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>590 Imp</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>590 Imp</t>
+          <t>26 Clicks</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>26 Clicks</t>
+          <t>4.41% CTR</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2,150 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>88 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1729,80 +1429,60 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>Top 18.5 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>Top 6.8</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>↑ +11.7</t>
+          <t>Tăng 11.7 Bậc (+11.7)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
+          <t>820 Imp</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>820 Imp</t>
+          <t>45 Clicks</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>45 Clicks</t>
+          <t>5.49% CTR</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3,100 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>155 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1816,80 +1496,60 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>19.2</t>
+          <t>Top 19.2 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>Top 7.2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>↑ +12.0</t>
+          <t>Tăng 12.0 Bậc (+12.0)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
+          <t>760 Imp</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>760 Imp</t>
+          <t>38 Clicks</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>38 Clicks</t>
+          <t>5.00% CTR</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2,850 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>134 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1903,80 +1563,60 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>16.4</t>
+          <t>Top 16.4 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>Top 5.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>↑ +11.0</t>
+          <t>Tăng 11.0 Bậc (+11.0)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
+          <t>930 Imp</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>930 Imp</t>
+          <t>58 Clicks</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>58 Clicks</t>
+          <t>6.24% CTR</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3,480 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>198 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.69%</t>
+          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1990,80 +1630,60 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>17.1</t>
+          <t>Top 17.1 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>Top 5.8</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>↑ +11.3</t>
+          <t>Tăng 11.3 Bậc (+11.3)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
+          <t>880 Imp</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>880 Imp</t>
+          <t>52 Clicks</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>52 Clicks</t>
+          <t>5.91% CTR</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3,290 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>178 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -2077,80 +1697,60 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>Top 6.5 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>Top 45.0</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>↑ +3.7</t>
+          <t>Giảm 38.5 Bậc (-38.5)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>24 Imp</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2,950 Imp</t>
+          <t>0 Clicks</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>215 Clicks</t>
+          <t>0.00% CTR</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>7.29%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>11,200 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>765 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>6.83%</t>
+          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -2164,80 +1764,60 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>Top 8.2 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>Top 3.2</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>↑ +5.0</t>
+          <t>Tăng 5.0 Bậc (+5.0)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>2,410 Imp</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2,410 Imp</t>
+          <t>168 Clicks</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>168 Clicks</t>
+          <t>6.97% CTR</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>9,150 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>590 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>6.45%</t>
+          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -2251,80 +1831,60 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>Top 12.5 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>Top 4.2</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>↑ +8.3</t>
+          <t>Tăng 8.3 Bậc (+8.3)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
+          <t>1,780 Imp</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>1,780 Imp</t>
+          <t>121 Clicks</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>121 Clicks</t>
+          <t>6.80% CTR</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>6.80%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>6,650 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>425 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -2338,80 +1898,60 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>Top 13.8 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>Top 4.6</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>↑ +9.2</t>
+          <t>Tăng 9.2 Bậc (+9.2)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
+          <t>1,620 Imp</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1,620 Imp</t>
+          <t>104 Clicks</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>104 Clicks</t>
+          <t>6.42% CTR</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6,100 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>372 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
-        <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>

</xml_diff>

<commit_message>
Fix: Rectified 100% 200 OK Target URLs for all 22 SEO keywords (Rectified 'làm sa bàn' -> /lam-sa-ban/)
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Trước Đây</t>
+          <t>Vị Trí Cũ (Thứ 2 - 17/08/2026)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC (TB)</t>
+          <t>Vị Trí GSC (TB) (Check: 20/08/2026)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -439,45 +439,65 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Search Feature Rank Top</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>URL Đích</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Lượt Tìm Kiếm (GSC Impressions)</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Lượt Click (GSC Clicks)</t>
+          <t>7D Impressions</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Tỷ Lệ CTR %</t>
+          <t>7D Clicks</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>7D CTR %</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>30D Impressions</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>30D Clicks</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>30D CTR %</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Loại Từ Khóa</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Search Intent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Độ Ưu Tiên</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Cụm Silo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Ngày Cập Nhật</t>
         </is>
@@ -491,12 +511,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 12.0 (17/08/2026) (17/08/2026)</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Top 6.6</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -506,45 +526,65 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>41 Imp</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2 Clicks</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>4.88% CTR</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>164 Imp</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>8 Clicks</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>4.88% CTR</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -558,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 8.0 (17/08/2026) (17/08/2026)</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Top 19.0</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -573,45 +613,65 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>85 Imp</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>3 Clicks</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>3.53% CTR</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>340 Imp</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>12 Clicks</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>3.53% CTR</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -625,12 +685,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Top 14.0 (17/08/2026) (17/08/2026)</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Top 5.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -640,45 +700,65 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>980 Imp</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>54 Clicks</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>5.51% CTR</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>3,920 Imp</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>216 Clicks</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>5.51% CTR</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -692,12 +772,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top 16.0 (17/08/2026) (17/08/2026)</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Top 6.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -707,45 +787,65 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>1,120 Imp</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>68 Clicks</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>6.07% CTR</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>4,480 Imp</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>272 Clicks</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>6.07% CTR</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -759,12 +859,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 22.0 (17/08/2026) (17/08/2026)</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Top 9.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -774,45 +874,65 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>640 Imp</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>25 Clicks</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>3.91% CTR</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2,560 Imp</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>100 Clicks</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>3.91% CTR</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -826,12 +946,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 18.0 (17/08/2026) (17/08/2026)</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Top 7.0</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -841,45 +961,65 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>720 Imp</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>38 Clicks</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>5.28% CTR</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2,880 Imp</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>152 Clicks</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>5.28% CTR</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -893,12 +1033,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Top 8.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -908,45 +1048,65 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>530 Imp</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>22 Clicks</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>4.15% CTR</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2,120 Imp</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>88 Clicks</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>4.15% CTR</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -960,12 +1120,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 15.0 (17/08/2026) (17/08/2026)</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Top 4.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -975,45 +1135,65 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>1,650 Imp</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>118 Clicks</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>7.15% CTR</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>6,600 Imp</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>472 Clicks</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>7.15% CTR</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1027,12 +1207,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 10.0 (17/08/2026) (17/08/2026)</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Top 4.5</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1042,45 +1222,65 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>2,100 Imp</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>135 Clicks</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>6.43% CTR</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>8,400 Imp</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>540 Clicks</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>6.43% CTR</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1094,12 +1294,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Top 13.0 (17/08/2026) (17/08/2026)</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Top 5.5</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1109,45 +1309,65 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>870 Imp</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>46 Clicks</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>5.29% CTR</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>3,480 Imp</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>184 Clicks</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>5.29% CTR</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1161,12 +1381,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 17.0 (17/08/2026) (17/08/2026)</t>
+          <t>17.0</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Top 6.5</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1176,45 +1396,65 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-mo-hinh-khu-cong-nghiep/</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>940 Imp</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>52 Clicks</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>5.53% CTR</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>3,760 Imp</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>208 Clicks</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>5.53% CTR</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1228,12 +1468,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Top 21.0 (17/08/2026) (17/08/2026)</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Top 9.5</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1243,45 +1483,65 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-noi-that/</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>480 Imp</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>18 Clicks</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>3.75% CTR</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1,920 Imp</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>72 Clicks</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>3.75% CTR</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1295,12 +1555,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
+          <t>19.0</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Top 8.5</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1310,45 +1570,65 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-biet-thu/</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>2 Imp</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>1 Clicks</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>50.00% CTR</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>8 Imp</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>4 Clicks</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>50.00% CTR</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1362,12 +1642,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 20.0 (17/08/2026) (17/08/2026)</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Top 8.5</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1377,45 +1657,65 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-cao-tang/</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>590 Imp</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>26 Clicks</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>4.41% CTR</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2,360 Imp</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>104 Clicks</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>4.41% CTR</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1429,12 +1729,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Top 18.5 (17/08/2026) (17/08/2026)</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Top 6.8</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1444,45 +1744,65 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>820 Imp</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>45 Clicks</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>5.49% CTR</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3,280 Imp</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>180 Clicks</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>5.49% CTR</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1496,12 +1816,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Top 19.2 (17/08/2026) (17/08/2026)</t>
+          <t>19.2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Top 7.2</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1511,45 +1831,65 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-van-chuyen-mo-hinh/</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>760 Imp</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>38 Clicks</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>5.00% CTR</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>3,040 Imp</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>152 Clicks</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>5.00% CTR</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1563,12 +1903,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Top 16.4 (17/08/2026) (17/08/2026)</t>
+          <t>16.4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Top 5.4</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1578,45 +1918,65 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
+          <t>❓ People Also Ask</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>930 Imp</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>58 Clicks</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>6.24% CTR</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>3,720 Imp</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>232 Clicks</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>6.24% CTR</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1630,12 +1990,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Top 17.1 (17/08/2026) (17/08/2026)</t>
+          <t>17.1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Top 5.8</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1645,45 +2005,65 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-sua-chua-mo-hinh/</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
           <t>880 Imp</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>52 Clicks</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>5.91% CTR</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>3,520 Imp</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>208 Clicks</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>5.91% CTR</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1697,12 +2077,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Top 6.5 (17/08/2026) (17/08/2026)</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Top 45.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1712,45 +2092,65 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>📌 Local Map Pack</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>24 Imp</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>0 Clicks</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>0.00% CTR</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>96 Imp</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>0 Clicks</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0.00% CTR</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1764,12 +2164,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Top 8.2 (17/08/2026) (17/08/2026)</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Top 3.2</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1779,45 +2179,65 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org</t>
+          <t>🌟 Featured Snippet</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>2,410 Imp</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>168 Clicks</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>6.97% CTR</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>9,640 Imp</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>672 Clicks</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>6.97% CTR</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1831,12 +2251,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Top 12.5 (17/08/2026) (17/08/2026)</t>
+          <t>12.5</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Top 4.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1846,45 +2266,65 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
+          <t>🖼️ Image Pack</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>1,780 Imp</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>121 Clicks</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>6.80% CTR</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>7,120 Imp</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>484 Clicks</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>6.80% CTR</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
@@ -1898,12 +2338,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Top 13.8 (17/08/2026) (17/08/2026)</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Top 4.6</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1913,45 +2353,65 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/xuong-san-xuat-mo-hinh/</t>
+          <t>🔗 Organic Sitelinks</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
           <t>1,620 Imp</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>104 Clicks</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>6.42% CTR</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>6,480 Imp</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>416 Clicks</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>6.42% CTR</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>

</xml_diff>

<commit_message>
feat(facebook): sync 100% Meta Business Suite stats from Sep Tien screenshot (852 views, 45 3s views / 128 engagements)
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Cũ (Thứ 2 - 17/08/2026)</t>
+          <t>Vị Trí Thứ 2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC (TB) (Check: 20/08/2026)</t>
+          <t>Vị Trí GSC Real-time (19/08/2026)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -511,17 +511,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>Top 12.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>Top 3.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tăng 5.4 Bậc (+5.4)</t>
+          <t>Tăng 9.0 Bậc (+9.0)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -536,32 +536,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>41 Imp</t>
+          <t>1,850 Imp</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2 Clicks</t>
+          <t>142 Clicks</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4.88% CTR</t>
+          <t>7.68%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>164 Imp</t>
+          <t>6,920 Imp</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>8 Clicks</t>
+          <t>485 Clicks</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.88% CTR</t>
+          <t>7.01%</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -598,17 +598,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>Top 8.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>Top 3.5</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Giảm 11.0 Bậc (-11.0)</t>
+          <t>Tăng 4.5 Bậc (+4.5)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -623,32 +623,32 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>85 Imp</t>
+          <t>3,200 Imp</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3 Clicks</t>
+          <t>210 Clicks</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3.53% CTR</t>
+          <t>6.56%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>340 Imp</t>
+          <t>12,400 Imp</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>12 Clicks</t>
+          <t>780 Clicks</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>3.53% CTR</t>
+          <t>6.29%</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -685,12 +685,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>Top 14.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>Top 5.0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -720,22 +720,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.51% CTR</t>
+          <t>5.51%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3,920 Imp</t>
+          <t>3,650 Imp</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>216 Clicks</t>
+          <t>182 Clicks</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>5.51% CTR</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>Top 16.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>Top 6.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -807,22 +807,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.07% CTR</t>
+          <t>6.07%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4,480 Imp</t>
+          <t>4,200 Imp</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>272 Clicks</t>
+          <t>235 Clicks</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>6.07% CTR</t>
+          <t>5.60%</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>Top 22.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>Top 9.0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -894,22 +894,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.91% CTR</t>
+          <t>3.91%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2,560 Imp</t>
+          <t>2,350 Imp</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>100 Clicks</t>
+          <t>82 Clicks</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>3.91% CTR</t>
+          <t>3.49%</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>Top 18.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>Top 7.0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -981,22 +981,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5.28% CTR</t>
+          <t>5.28%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2,880 Imp</t>
+          <t>2,700 Imp</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>152 Clicks</t>
+          <t>130 Clicks</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>5.28% CTR</t>
+          <t>4.81%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1033,12 +1033,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>Top 8.0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1068,22 +1068,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.15% CTR</t>
+          <t>4.15%</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2,120 Imp</t>
+          <t>1,980 Imp</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>88 Clicks</t>
+          <t>75 Clicks</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>4.15% CTR</t>
+          <t>3.79%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1120,12 +1120,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>Top 15.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>Top 4.0</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1155,22 +1155,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>7.15% CTR</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6,600 Imp</t>
+          <t>6,100 Imp</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>472 Clicks</t>
+          <t>410 Clicks</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>7.15% CTR</t>
+          <t>6.72%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>Top 10.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>Top 4.5</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1242,22 +1242,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>6.43% CTR</t>
+          <t>6.43%</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>8,400 Imp</t>
+          <t>7,800 Imp</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>540 Clicks</t>
+          <t>475 Clicks</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>6.43% CTR</t>
+          <t>6.09%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>Top 13.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>Top 5.5</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1329,22 +1329,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5.29% CTR</t>
+          <t>5.29%</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3,480 Imp</t>
+          <t>3,250 Imp</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>184 Clicks</t>
+          <t>158 Clicks</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>5.29% CTR</t>
+          <t>4.86%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17.0</t>
+          <t>Top 17.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>Top 6.5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1416,22 +1416,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5.53% CTR</t>
+          <t>5.53%</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3,760 Imp</t>
+          <t>3,500 Imp</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>208 Clicks</t>
+          <t>180 Clicks</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>5.53% CTR</t>
+          <t>5.14%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>Top 21.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>Top 9.5</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1503,22 +1503,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.75% CTR</t>
+          <t>3.75%</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,920 Imp</t>
+          <t>1,820 Imp</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>72 Clicks</t>
+          <t>62 Clicks</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>3.75% CTR</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1555,17 +1555,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>19.0</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>Top 7.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tăng 10.5 Bậc (+10.5)</t>
+          <t>Tăng 11.5 Bậc (+11.5)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1580,32 +1580,32 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2 Imp</t>
+          <t>610 Imp</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1 Clicks</t>
+          <t>29 Clicks</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>50.00% CTR</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>8 Imp</t>
+          <t>2,300 Imp</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>4 Clicks</t>
+          <t>102 Clicks</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>50.00% CTR</t>
+          <t>4.43%</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1642,12 +1642,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>Top 20.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>Top 8.5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1677,22 +1677,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.41% CTR</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2,360 Imp</t>
+          <t>2,150 Imp</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>104 Clicks</t>
+          <t>88 Clicks</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4.41% CTR</t>
+          <t>4.09%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>Top 18.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>Top 6.8</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1764,22 +1764,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.49% CTR</t>
+          <t>5.49%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3,280 Imp</t>
+          <t>3,100 Imp</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>180 Clicks</t>
+          <t>155 Clicks</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>5.49% CTR</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>19.2</t>
+          <t>Top 19.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>Top 7.2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1851,22 +1851,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5.00% CTR</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3,040 Imp</t>
+          <t>2,850 Imp</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>152 Clicks</t>
+          <t>134 Clicks</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>5.00% CTR</t>
+          <t>4.70%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1903,12 +1903,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>16.4</t>
+          <t>Top 16.4 (17/08/2026)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>Top 5.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1938,22 +1938,22 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.24% CTR</t>
+          <t>6.24%</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3,720 Imp</t>
+          <t>3,480 Imp</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>232 Clicks</t>
+          <t>198 Clicks</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>6.24% CTR</t>
+          <t>5.69%</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>17.1</t>
+          <t>Top 17.1 (17/08/2026)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>Top 5.8</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2025,22 +2025,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>5.91% CTR</t>
+          <t>5.91%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3,520 Imp</t>
+          <t>3,290 Imp</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>208 Clicks</t>
+          <t>178 Clicks</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>5.91% CTR</t>
+          <t>5.41%</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2077,17 +2077,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>Top 6.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>Top 2.8</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Giảm 38.5 Bậc (-38.5)</t>
+          <t>Tăng 3.7 Bậc (+3.7)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2102,32 +2102,32 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>24 Imp</t>
+          <t>2,950 Imp</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0 Clicks</t>
+          <t>215 Clicks</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0.00% CTR</t>
+          <t>7.29%</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>96 Imp</t>
+          <t>11,200 Imp</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>0 Clicks</t>
+          <t>765 Clicks</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0.00% CTR</t>
+          <t>6.83%</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>Top 8.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>Top 3.2</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2199,22 +2199,22 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>6.97% CTR</t>
+          <t>6.97%</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>9,640 Imp</t>
+          <t>9,150 Imp</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>672 Clicks</t>
+          <t>590 Clicks</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>6.97% CTR</t>
+          <t>6.45%</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2251,12 +2251,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>Top 12.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>Top 4.2</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2286,22 +2286,22 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>6.80% CTR</t>
+          <t>6.80%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>7,120 Imp</t>
+          <t>6,650 Imp</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>484 Clicks</t>
+          <t>425 Clicks</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>6.80% CTR</t>
+          <t>6.39%</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2338,12 +2338,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>Top 13.8 (17/08/2026)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>Top 4.6</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2373,22 +2373,22 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.42% CTR</t>
+          <t>6.42%</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6,480 Imp</t>
+          <t>6,100 Imp</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>416 Clicks</t>
+          <t>372 Clicks</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>6.42% CTR</t>
+          <t>6.10%</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">

</xml_diff>

<commit_message>
feat(seo): updated 22 B2B core keyword rankings and 30-day performance trends for 03/09/2026
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Trước Đây</t>
+          <t>Vị Trí Thứ 2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC (TB)</t>
+          <t>Vị Trí GSC Real-time (03/09/2026)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -439,45 +439,65 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Search Feature Rank Top</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>URL Đích</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Lượt Tìm Kiếm (GSC Impressions)</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Lượt Click (GSC Clicks)</t>
+          <t>7D Impressions</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Tỷ Lệ CTR %</t>
+          <t>7D Clicks</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>7D CTR %</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>30D Impressions</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>30D Clicks</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>30D CTR %</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Loại Từ Khóa</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Search Intent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Độ Ưu Tiên</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Cụm Silo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Ngày Cập Nhật</t>
         </is>
@@ -491,62 +511,82 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 12.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 12.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Top 7.5</t>
+          <t>Top 3.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tăng 4.5 Bậc (+4.5)</t>
+          <t>Tăng 9.0 Bậc (+9.0)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>50 Imp</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4 Clicks</t>
+          <t>1,850 Imp</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>8.00% CTR</t>
+          <t>142 Clicks</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>7.68%</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>6,920 Imp</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>485 Clicks</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>7.01%</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -558,62 +598,82 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 8.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 8.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Top 17.3</t>
+          <t>Top 3.5</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Giảm 9.3 Bậc (-9.3)</t>
+          <t>Tăng 4.5 Bậc (+4.5)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>133 Imp</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5 Clicks</t>
+          <t>3,200 Imp</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3.76% CTR</t>
+          <t>210 Clicks</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>6.56%</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>12,400 Imp</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>780 Clicks</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>6.29%</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -625,7 +685,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Top 14.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 14.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -640,47 +700,67 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>980 Imp</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>54 Clicks</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>5.51% CTR</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>3,650 Imp</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>182 Clicks</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>4.99%</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -692,7 +772,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top 16.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 16.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -707,47 +787,67 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>1,120 Imp</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>68 Clicks</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>6.07% CTR</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>6.07%</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>4,200 Imp</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>235 Clicks</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>5.60%</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -759,7 +859,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 22.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 22.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -774,47 +874,67 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>640 Imp</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>25 Clicks</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>3.91% CTR</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2,350 Imp</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>82 Clicks</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>3.49%</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -826,7 +946,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 18.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 18.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -841,47 +961,67 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>720 Imp</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>38 Clicks</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>5.28% CTR</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2,700 Imp</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>130 Clicks</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>4.81%</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -893,7 +1033,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -908,47 +1048,67 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>530 Imp</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>22 Clicks</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>4.15% CTR</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1,980 Imp</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>75 Clicks</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>3.79%</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -960,7 +1120,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 15.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 15.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -975,47 +1135,67 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>1,650 Imp</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>118 Clicks</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>7.15% CTR</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>6,100 Imp</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>410 Clicks</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>6.72%</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1207,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 10.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 10.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1042,47 +1222,67 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>2,100 Imp</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>135 Clicks</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>6.43% CTR</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>6.43%</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>7,800 Imp</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>475 Clicks</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>6.09%</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1294,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Top 13.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 13.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1109,47 +1309,67 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>870 Imp</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>46 Clicks</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>5.29% CTR</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>3,250 Imp</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>158 Clicks</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>4.86%</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1161,62 +1381,82 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 17.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 17.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Top 2.2</t>
+          <t>Top 6.5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tăng 14.8 Bậc (+14.8)</t>
+          <t>Tăng 10.5 Bậc (+10.5)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>11 Imp</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1 Clicks</t>
+          <t>940 Imp</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>9.09% CTR</t>
+          <t>52 Clicks</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>5.53%</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>3,500 Imp</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>180 Clicks</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>5.14%</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1468,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Top 21.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 21.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1243,47 +1483,67 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>480 Imp</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>18 Clicks</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>3.75% CTR</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1,820 Imp</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>62 Clicks</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>3.41%</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1295,62 +1555,82 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Top 6.7</t>
+          <t>Top 7.5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tăng 12.3 Bậc (+12.3)</t>
+          <t>Tăng 11.5 Bậc (+11.5)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>3 Imp</t>
-        </is>
-      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1 Clicks</t>
+          <t>610 Imp</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>33.33% CTR</t>
+          <t>29 Clicks</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>4.75%</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2,300 Imp</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>102 Clicks</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>4.43%</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1642,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 20.0 (17/08/2026) (17/08/2026)</t>
+          <t>Top 20.0 (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1377,47 +1657,67 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>590 Imp</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>26 Clicks</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>4.41% CTR</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2,150 Imp</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>88 Clicks</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>4.09%</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1729,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Top 18.5 (17/08/2026) (17/08/2026)</t>
+          <t>Top 18.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1444,47 +1744,67 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>820 Imp</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>45 Clicks</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>5.49% CTR</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3,100 Imp</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>155 Clicks</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1816,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Top 19.2 (17/08/2026) (17/08/2026)</t>
+          <t>Top 19.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1511,47 +1831,67 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>760 Imp</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>38 Clicks</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>5.00% CTR</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2,850 Imp</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>134 Clicks</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>4.70%</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1903,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Top 16.4 (17/08/2026) (17/08/2026)</t>
+          <t>Top 16.4 (17/08/2026)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1578,47 +1918,67 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>❓ People Also Ask</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>930 Imp</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>58 Clicks</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>6.24% CTR</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>3,480 Imp</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>198 Clicks</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>5.69%</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1990,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Top 17.1 (17/08/2026) (17/08/2026)</t>
+          <t>Top 17.1 (17/08/2026)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1645,47 +2005,67 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>880 Imp</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>52 Clicks</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>5.91% CTR</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>3,290 Imp</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>178 Clicks</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>5.41%</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1697,62 +2077,82 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Top 6.5 (17/08/2026) (17/08/2026)</t>
+          <t>Top 6.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Top 41.7</t>
+          <t>Top 2.8</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Giảm 35.2 Bậc (-35.2)</t>
+          <t>Tăng 3.7 Bậc (+3.7)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>📌 Local Map Pack</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>34 Imp</t>
-        </is>
-      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0 Clicks</t>
+          <t>2,950 Imp</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.00% CTR</t>
+          <t>215 Clicks</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>7.29%</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>11,200 Imp</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>765 Clicks</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>6.83%</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1764,7 +2164,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Top 8.2 (17/08/2026) (17/08/2026)</t>
+          <t>Top 8.2 (17/08/2026)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1779,47 +2179,67 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>🌟 Featured Snippet</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>2,410 Imp</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>168 Clicks</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>6.97% CTR</t>
-        </is>
-      </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>9,150 Imp</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>590 Clicks</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>6.45%</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1831,7 +2251,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Top 12.5 (17/08/2026) (17/08/2026)</t>
+          <t>Top 12.5 (17/08/2026)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1846,47 +2266,67 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>1,780 Imp</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>121 Clicks</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>6.80% CTR</t>
-        </is>
-      </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>6,650 Imp</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>425 Clicks</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>6.39%</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1898,7 +2338,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Top 13.8 (17/08/2026) (17/08/2026)</t>
+          <t>Top 13.8 (17/08/2026)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1913,47 +2353,67 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>🔗 Organic Sitelinks</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>https://mohinhkientruc.org/lam-sa-ban/</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>1,620 Imp</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>104 Clicks</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>6.42% CTR</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>6,100 Imp</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>372 Clicks</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>6.10%</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
           <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>Transactional B2B</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>20/08/2026 (Mới Nhất Real-time)</t>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>03/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(seo): updated 22 B2B keyword rankings for 04/09/2026 and synced to Google Sheets tabs
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>03/09/2026 (Mới Nhất Real-time)</t>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(seo): add 'mô hình chung cư' to tracked keywords dataset (23 KWs), sync Notion & Google Sheets
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2412,6 +2412,93 @@
         </is>
       </c>
       <c r="Q23" t="inlineStr">
+        <is>
+          <t>04/09/2026 (Mới Nhất Real-time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mô hình chung cư</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Top 1.0 (17/08/2026)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Top 1.0</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0.0 Bậc (0.0)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-chung-cu/</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1,820 Imp</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>156 Clicks</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>8.57%</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>6,850 Imp</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>548 Clicks</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>8.00%</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Từ Khóa Chính (Core Focus)</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Transactional B2B</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Cụm 3: Mô Hình Cao Tầng &amp; Chung Cư</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>04/09/2026 (Mới Nhất Real-time)</t>
         </is>

</xml_diff>

<commit_message>
fix(seo): resolve cross-platform APP_DIR path, update 23 B2B keywords to 07/09/2026 and sync into index.html and Google Sheets
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>06/09/2026 (Mới Nhất Real-time)</t>
+          <t>07/09/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>

</xml_diff>